<commit_message>
feat: establish complete OBE-based curriculum documentation and supporting automation tools for SISTEKIN 2026
</commit_message>
<xml_diff>
--- a/KURIKULUM2026_REVISI/001_ANALISIS_VMTS_DAN_POSITIONING_STRATEGIS_SISTEKIN.xlsx
+++ b/KURIKULUM2026_REVISI/001_ANALISIS_VMTS_DAN_POSITIONING_STRATEGIS_SISTEKIN.xlsx
@@ -1,175 +1,93 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\!!MYDOCUMENTS2026\!!!SISTEKIN2026\!!BRAINSTORMING_KURIKULUM2026\KURIKULUM2026_REVISI\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{611B7657-25E2-48A7-8014-54F454C74252}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Data" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
-  <si>
-    <t>SISTEKIN 2026 — 001_ANALISIS_VMTS_DAN_POSITIONING_STRATEGIS_SISTEKIN</t>
-  </si>
-  <si>
-    <t>Dokumen Kurikulum KPT-OBE SISTEKIN 2026</t>
-  </si>
-  <si>
-    <t>2. DISTINCTIVE POSITIONING (KEKHASAN DAN KEUNGGULAN STRATEGIS)</t>
-  </si>
-  <si>
-    <t>Program Studi</t>
-  </si>
-  <si>
-    <t>Fokus Utama Keilmuan &amp; Peran Kompetensi</t>
-  </si>
-  <si>
-    <t>**Teknik Informatika / Ilmu Komputer**</t>
-  </si>
-  <si>
-    <t>Teori komputasi, algoritma fundamental murni, arsitektur internal perangkat keras, serta riset model matematika kecerdasan buatan.</t>
-  </si>
-  <si>
-    <t>**SISTEKIN (Sistem &amp; Teknologi Informasi)**</t>
-  </si>
-  <si>
-    <t>**PEREKAYASA &amp; PENGINTEGRASI SISTEM CERDAS NYATA (AI Integrator):** Mengintegrasikan model AI, infrastruktur cloud &amp; IoT, keamanan siber, dan platform digital ke dalam proses bisnis dan organisasi dengan semangat kemandirian Technopreneurship.</t>
-  </si>
-  <si>
-    <t>**Bisnis Digital / Manajemen**</t>
-  </si>
-  <si>
-    <t>Strategi pemasaran digital, model finansial, operasional bisnis, dan manajemen e-commerce (tanpa fokus pada rekayasa kode/infra).</t>
-  </si>
-  <si>
-    <t>3. ENVIRONMENTAL SCANNING &amp; ANALISIS SWOT (LAM INFOKOM KRITERIA 1)</t>
-  </si>
-  <si>
-    <t>STRENGTHS (Kekuatan Internal)</t>
-  </si>
-  <si>
-    <t>WEAKNESSES (Kelemahan Internal)</t>
-  </si>
-  <si>
-    <t>1. Kurikulum modern berbasis OBE terkini (APTIKOM v2.0, IS2020, IT2017).&lt;br&gt;2. Visi keilmuan yang sangat fokus dan relevan: AI Integration &amp; Technopreneurship.&lt;br&gt;3. Paket SKS terstruktur (146 SKS / 55 MK) dengan 3 peminatan seimbang.&lt;br&gt;4. Adanya pilar Capstone &amp; opsi Tugas Akhir non-skripsi.</t>
-  </si>
-  <si>
-    <t>1. Status program studi baru yang belum memiliki rekam jejak alumni (*tracer study*).&lt;br&gt;2. Kebutuhan peningkatan kapasitas dosen dalam sertifikasi industri bertaraf global.&lt;br&gt;3. Fasilitas laboratorium spesialisasi cerdas yang sedang dalam proses akselerasi.</t>
-  </si>
-  <si>
-    <t>**OPPORTUNITIES (Peluang Eksternal)**</t>
-  </si>
-  <si>
-    <t>**THREATS (Ancaman Eksternal)**</t>
-  </si>
-  <si>
-    <t>1. Lonjakan kebutuhan industri terhadap Data/AI Engineer &amp; Cloud Architect.&lt;br&gt;2. Kebijakan Permendikbudristek 53/2023 yang memberi fleksibilitas MBKM &amp; TA.&lt;br&gt;3. Kemitraan strategis Malang Raya sebagai kota pendidikan &amp; hub digital.</t>
-  </si>
-  <si>
-    <t>1. Kecepatan disrupsi teknologi AI generatif yang dapat mengusir kurikulum usang.&lt;br&gt;2. Persaingan ketat dengan prodi TI/SI konvensional dari PTN/PTS mapan.&lt;br&gt;3. Standar kompetensi industri yang menuntut penguasaan sertifikasi internasional.</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="6">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
       <sz val="13"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <color rgb="00FFFFFF"/>
       <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
     </font>
     <font>
-      <b/>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
       <sz val="10"/>
-      <color rgb="FF1F3864"/>
-      <name val="Calibri"/>
     </font>
     <font>
-      <b/>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
       <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <color rgb="00000000"/>
       <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1F3864"/>
+        <fgColor rgb="001F3864"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFBDD7EE"/>
+        <fgColor rgb="00BDD7EE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF2E75B6"/>
+        <fgColor rgb="002E75B6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEEF4FB"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
+        <fgColor rgb="00EEF4FB"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -179,40 +97,59 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFB8CCE4"/>
+        <color rgb="00B8CCE4"/>
       </left>
       <right style="thin">
-        <color rgb="FFB8CCE4"/>
+        <color rgb="00B8CCE4"/>
       </right>
       <top style="thin">
-        <color rgb="FFB8CCE4"/>
+        <color rgb="00B8CCE4"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFB8CCE4"/>
+        <color rgb="00B8CCE4"/>
       </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00B8CCE4"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B8CCE4"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B8CCE4"/>
+      </top>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
       <left/>
       <right/>
       <top style="thin">
-        <color rgb="FFB8CCE4"/>
+        <color rgb="00B8CCE4"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFB8CCE4"/>
+        <color rgb="00B8CCE4"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left/>
       <right style="thin">
-        <color rgb="FFB8CCE4"/>
+        <color rgb="00B8CCE4"/>
       </right>
       <top style="thin">
-        <color rgb="FFB8CCE4"/>
+        <color rgb="00B8CCE4"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFB8CCE4"/>
+        <color rgb="00B8CCE4"/>
       </bottom>
       <diagonal/>
     </border>
@@ -220,46 +157,101 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+  <cellXfs count="9">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -547,119 +539,156 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="FF1F3864"/>
+    <tabColor rgb="001F3864"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="2" width="69" customWidth="1"/>
-    <col min="3" max="6" width="10" customWidth="1"/>
+    <col width="69" customWidth="1" min="1" max="1"/>
+    <col width="69" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="6"/>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A6" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="6"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="B12" s="10" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>19</v>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>SISTEKIN 2026 — 001_ANALISIS_VMTS_DAN_POSITIONING_STRATEGIS_SISTEKIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Dokumen Kurikulum KPT-OBE SISTEKIN 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>2. DISTINCTIVE POSITIONING (KEKHASAN DAN KEUNGGULAN STRATEGIS)</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n"/>
+      <c r="C3" s="4" t="n"/>
+      <c r="D3" s="4" t="n"/>
+      <c r="E3" s="4" t="n"/>
+      <c r="F3" s="5" t="n"/>
+    </row>
+    <row r="4" ht="26" customHeight="1">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Program Studi</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Fokus Utama Keilmuan &amp; Peran Kompetensi</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>**Teknik Informatika / Ilmu Komputer**</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Teori komputasi, algoritma fundamental murni, arsitektur internal perangkat keras, serta riset model matematika kecerdasan buatan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>**SISTEKIN (Sistem &amp; Teknologi Informasi)**</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>**PEREKAYASA &amp; PENGINTEGRASI SISTEM CERDAS NYATA (AI Integrator):** Mengintegrasikan model AI, infrastruktur cloud &amp; IoT, keamanan siber, dan platform digital ke dalam proses bisnis dan organisasi dengan semangat kemandirian Technopreneurship.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="16" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>**Bisnis Digital / Manajemen**</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Strategi pemasaran digital, model finansial, operasional bisnis, dan manajemen e-commerce (tanpa fokus pada rekayasa kode/infra).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>3. ENVIRONMENTAL SCANNING &amp; ANALISIS SWOT (LAM INFOKOM KRITERIA 1)</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n"/>
+      <c r="C9" s="4" t="n"/>
+      <c r="D9" s="4" t="n"/>
+      <c r="E9" s="4" t="n"/>
+      <c r="F9" s="5" t="n"/>
+    </row>
+    <row r="10" ht="26" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>STRENGTHS (Kekuatan Internal)</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>WEAKNESSES (Kelemahan Internal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="16" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>1. Kurikulum modern berbasis OBE terkini (APTIKOM v2.0, IS2020, IT2017).&lt;br&gt;2. Visi keilmuan yang sangat fokus dan relevan: AI Integration &amp; Technopreneurship.&lt;br&gt;3. Paket SKS terstruktur (146 SKS / 55 MK) dengan 3 peminatan seimbang.&lt;br&gt;4. Adanya pilar Capstone &amp; opsi Tugas Akhir non-skripsi.</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>1. Status program studi baru yang belum memiliki rekam jejak alumni (*tracer study*).&lt;br&gt;2. Kebutuhan peningkatan kapasitas dosen dalam sertifikasi industri bertaraf global.&lt;br&gt;3. Fasilitas laboratorium spesialisasi cerdas yang sedang dalam proses akselerasi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>**OPPORTUNITIES (Peluang Eksternal)**</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>**THREATS (Ancaman Eksternal)**</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="16" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>1. Lonjakan kebutuhan industri terhadap Data/AI Engineer &amp; Cloud Architect.&lt;br&gt;2. Kebijakan Permendikbudristek 53/2023 yang memberi fleksibilitas MBKM &amp; TA.&lt;br&gt;3. Kemitraan strategis Malang Raya sebagai kota pendidikan &amp; hub digital.</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>1. Kecepatan disrupsi teknologi AI generatif yang dapat mengusir kurikulum usang.&lt;br&gt;2. Persaingan ketat dengan prodi TI/SI konvensional dari PTN/PTS mapan.&lt;br&gt;3. Standar kompetensi industri yang menuntut penguasaan sertifikasi internasional.</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -670,6 +699,5 @@
     <mergeCell ref="A9:F9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>